<commit_message>
fix(format): Document used normal format enum
XLCellsUsedOptions.NormalFormats wasn't propertly described.

As far as I can tell from original code before style rework, this is intended meaning behind the used format. It is also qute natural one. The other possible choice is to say cell format is different from default format, but that would mean a changing a format of a column would make all cells in a column markes as used, depite not being materialized or anything.

The quote doesn't get a special treatment, because inherited format can also have a quote and that gets inherited as everythign else. That might have made sense before cell had types value, not anymore.

The test files had some blank cells removed when style was same as the inherited one (e.g. <x:c r="A9" s="1"/> where column had s=1) and few others that had empty row <x:row r="2" spans="1:4"/> without any cells.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Sparklines/SampleSparklines.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Sparklines/SampleSparklines.xlsx
@@ -1548,7 +1548,6 @@
       </x:c>
     </x:row>
     <x:row r="3" spans="1:16">
-      <x:c r="A3" s="1"/>
       <x:c r="C3" s="0">
         <x:v>4</x:v>
       </x:c>
@@ -1593,7 +1592,6 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:16">
-      <x:c r="A4" s="1"/>
       <x:c r="C4" s="0">
         <x:v>6</x:v>
       </x:c>
@@ -1685,7 +1683,6 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:16">
-      <x:c r="A6" s="1"/>
       <x:c r="C6" s="0">
         <x:v>8</x:v>
       </x:c>
@@ -1730,7 +1727,6 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:16">
-      <x:c r="A7" s="1"/>
       <x:c r="C7" s="0">
         <x:v>10</x:v>
       </x:c>
@@ -1822,7 +1818,6 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:16">
-      <x:c r="A9" s="1"/>
       <x:c r="C9" s="0">
         <x:v>13</x:v>
       </x:c>
@@ -1867,7 +1862,6 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:16">
-      <x:c r="A10" s="1"/>
       <x:c r="C10" s="0">
         <x:v>14</x:v>
       </x:c>
@@ -1959,7 +1953,6 @@
       </x:c>
     </x:row>
     <x:row r="12" spans="1:16">
-      <x:c r="A12" s="1"/>
       <x:c r="C12" s="0">
         <x:v>17</x:v>
       </x:c>
@@ -2004,7 +1997,6 @@
       </x:c>
     </x:row>
     <x:row r="13" spans="1:16">
-      <x:c r="A13" s="1"/>
       <x:c r="C13" s="0">
         <x:v>18</x:v>
       </x:c>
@@ -2096,7 +2088,6 @@
       </x:c>
     </x:row>
     <x:row r="15" spans="1:16">
-      <x:c r="A15" s="1"/>
       <x:c r="C15" s="0">
         <x:v>21</x:v>
       </x:c>
@@ -2141,7 +2132,6 @@
       </x:c>
     </x:row>
     <x:row r="16" spans="1:16">
-      <x:c r="A16" s="1"/>
       <x:c r="C16" s="0">
         <x:v>23</x:v>
       </x:c>
@@ -2233,7 +2223,6 @@
       </x:c>
     </x:row>
     <x:row r="18" spans="1:16">
-      <x:c r="A18" s="1"/>
       <x:c r="C18" s="0">
         <x:v>25</x:v>
       </x:c>
@@ -2278,7 +2267,6 @@
       </x:c>
     </x:row>
     <x:row r="19" spans="1:16">
-      <x:c r="A19" s="1"/>
       <x:c r="C19" s="0">
         <x:v>27</x:v>
       </x:c>
@@ -2601,7 +2589,6 @@
       </x:c>
     </x:row>
     <x:row r="3" spans="1:16">
-      <x:c r="A3" s="1"/>
       <x:c r="C3" s="0">
         <x:v>4</x:v>
       </x:c>
@@ -2646,7 +2633,6 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:16">
-      <x:c r="A4" s="1"/>
       <x:c r="C4" s="0">
         <x:v>6</x:v>
       </x:c>
@@ -2738,7 +2724,6 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:16">
-      <x:c r="A6" s="1"/>
       <x:c r="C6" s="0">
         <x:v>8</x:v>
       </x:c>
@@ -2783,7 +2768,6 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:16">
-      <x:c r="A7" s="1"/>
       <x:c r="C7" s="0">
         <x:v>10</x:v>
       </x:c>
@@ -2875,7 +2859,6 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:16">
-      <x:c r="A9" s="1"/>
       <x:c r="C9" s="0">
         <x:v>13</x:v>
       </x:c>
@@ -2920,7 +2903,6 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:16">
-      <x:c r="A10" s="1"/>
       <x:c r="C10" s="0">
         <x:v>14</x:v>
       </x:c>
@@ -3012,7 +2994,6 @@
       </x:c>
     </x:row>
     <x:row r="12" spans="1:16">
-      <x:c r="A12" s="1"/>
       <x:c r="C12" s="0">
         <x:v>17</x:v>
       </x:c>
@@ -3057,7 +3038,6 @@
       </x:c>
     </x:row>
     <x:row r="13" spans="1:16">
-      <x:c r="A13" s="1"/>
       <x:c r="C13" s="0">
         <x:v>18</x:v>
       </x:c>
@@ -3149,7 +3129,6 @@
       </x:c>
     </x:row>
     <x:row r="15" spans="1:16">
-      <x:c r="A15" s="1"/>
       <x:c r="C15" s="0">
         <x:v>21</x:v>
       </x:c>
@@ -3194,7 +3173,6 @@
       </x:c>
     </x:row>
     <x:row r="16" spans="1:16">
-      <x:c r="A16" s="1"/>
       <x:c r="C16" s="0">
         <x:v>23</x:v>
       </x:c>
@@ -3286,7 +3264,6 @@
       </x:c>
     </x:row>
     <x:row r="18" spans="1:16">
-      <x:c r="A18" s="1"/>
       <x:c r="C18" s="0">
         <x:v>25</x:v>
       </x:c>
@@ -3331,7 +3308,6 @@
       </x:c>
     </x:row>
     <x:row r="19" spans="1:16">
-      <x:c r="A19" s="1"/>
       <x:c r="C19" s="0">
         <x:v>27</x:v>
       </x:c>

</xml_diff>